<commit_message>
Deployed 8e0e0593 to dev with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/dev/assets/coremeta4cat_vocabulary.xlsx
+++ b/dev/assets/coremeta4cat_vocabulary.xlsx
@@ -5985,7 +5985,7 @@
       <c r="H116" s="13" t="inlineStr"/>
       <c r="I116" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:hydrolysis_ratio</t>
+          <t>voc4cat:0008157</t>
         </is>
       </c>
       <c r="J116" s="13" t="inlineStr">
@@ -6113,7 +6113,7 @@
       <c r="H119" s="13" t="inlineStr"/>
       <c r="I119" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:surfactant_template</t>
+          <t>voc4cat:0008147</t>
         </is>
       </c>
       <c r="J119" s="13" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="I126" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:filling_volume</t>
+          <t>voc4cat:0008148</t>
         </is>
       </c>
       <c r="J126" s="13" t="inlineStr">
@@ -6494,7 +6494,7 @@
       <c r="H128" s="13" t="inlineStr"/>
       <c r="I128" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:cooling_rate</t>
+          <t>voc4cat:0008149</t>
         </is>
       </c>
       <c r="J128" s="13" t="inlineStr">
@@ -6936,7 +6936,7 @@
       <c r="H139" s="16" t="inlineStr"/>
       <c r="I139" s="16" t="inlineStr">
         <is>
-          <t>coremeta4cat:PlasmaAssisted</t>
+          <t>voc4cat:0008152</t>
         </is>
       </c>
       <c r="J139" s="16" t="inlineStr">
@@ -6981,7 +6981,7 @@
       <c r="H140" s="13" t="inlineStr"/>
       <c r="I140" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:plasma_type</t>
+          <t>voc4cat:0008153</t>
         </is>
       </c>
       <c r="J140" s="13" t="inlineStr">
@@ -7029,7 +7029,7 @@
       <c r="H141" s="13" t="inlineStr"/>
       <c r="I141" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:power_input</t>
+          <t>voc4cat:0008154</t>
         </is>
       </c>
       <c r="J141" s="13" t="inlineStr">
@@ -7113,7 +7113,7 @@
       <c r="H143" s="13" t="inlineStr"/>
       <c r="I143" s="13" t="inlineStr">
         <is>
-          <t>coremeta4cat:exposure_time</t>
+          <t>voc4cat:0008155</t>
         </is>
       </c>
       <c r="J143" s="13" t="inlineStr">
@@ -7489,7 +7489,7 @@
       <c r="H152" s="16" t="inlineStr"/>
       <c r="I152" s="16" t="inlineStr">
         <is>
-          <t>coremeta4cat:CombustionSynthesis</t>
+          <t>voc4cat:0008156</t>
         </is>
       </c>
       <c r="J152" s="16" t="inlineStr">

</xml_diff>

<commit_message>
Deployed e112eb79 to dev with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/dev/assets/coremeta4cat_vocabulary.xlsx
+++ b/dev/assets/coremeta4cat_vocabulary.xlsx
@@ -1591,7 +1591,7 @@
       <c r="H4" s="11" t="inlineStr"/>
       <c r="I4" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008105</t>
+          <t>voc4cat:0008105</t>
         </is>
       </c>
       <c r="J4" s="11" t="inlineStr">
@@ -1631,7 +1631,7 @@
       <c r="H5" s="13" t="inlineStr"/>
       <c r="I5" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008104</t>
+          <t>voc4cat:0008104</t>
         </is>
       </c>
       <c r="J5" s="13" t="inlineStr">
@@ -1675,7 +1675,7 @@
       <c r="H6" s="13" t="inlineStr"/>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007246</t>
+          <t>voc4cat:0007246</t>
         </is>
       </c>
       <c r="J6" s="13" t="inlineStr">
@@ -2327,7 +2327,7 @@
       <c r="H23" s="16" t="inlineStr"/>
       <c r="I23" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000122</t>
+          <t>voc4cat:0000122</t>
         </is>
       </c>
       <c r="J23" s="16" t="inlineStr">
@@ -2444,7 +2444,7 @@
       <c r="H26" s="16" t="inlineStr"/>
       <c r="I26" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007794</t>
+          <t>voc4cat:0007794</t>
         </is>
       </c>
       <c r="J26" s="16" t="inlineStr">
@@ -2493,7 +2493,7 @@
       <c r="H27" s="12" t="inlineStr"/>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008118</t>
+          <t>voc4cat:0008118</t>
         </is>
       </c>
       <c r="J27" s="12" t="inlineStr">
@@ -3144,7 +3144,7 @@
         <is>
           <t>A MaterialSample that is the product of a catalyst Synthesis.
 The specific type of catalyst (e.g. heterogeneous, supported metal)
-is expressed via rdf_type using a VOC4CAT term.</t>
+is expressed via rdf_type using a voc4cat term.</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       <c r="H54" s="16" t="inlineStr"/>
       <c r="I54" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007016</t>
+          <t>voc4cat:0007016</t>
         </is>
       </c>
       <c r="J54" s="16" t="inlineStr">
@@ -3537,7 +3537,7 @@
 method-specific parameters. Linked from Synthesis via realized_plan.
 The specific preparation method type should additionally be expressed
 via rdf_type on the Synthesis activity using a voc4cat term
-(e.g. VOC4CAT:0007016 for preparation method).</t>
+(e.g. voc4cat:0007016 for preparation method).</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3600,7 @@
       <c r="H56" s="16" t="inlineStr"/>
       <c r="I56" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007028</t>
+          <t>voc4cat:0007028</t>
         </is>
       </c>
       <c r="J56" s="16" t="inlineStr">
@@ -3645,7 +3645,7 @@
       <c r="H57" s="13" t="inlineStr"/>
       <c r="I57" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008119</t>
+          <t>voc4cat:0008119</t>
         </is>
       </c>
       <c r="J57" s="13" t="inlineStr">
@@ -3693,7 +3693,7 @@
       <c r="H58" s="13" t="inlineStr"/>
       <c r="I58" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008120</t>
+          <t>voc4cat:0008120</t>
         </is>
       </c>
       <c r="J58" s="13" t="inlineStr">
@@ -3777,7 +3777,7 @@
       <c r="H60" s="13" t="inlineStr"/>
       <c r="I60" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008121</t>
+          <t>voc4cat:0008121</t>
         </is>
       </c>
       <c r="J60" s="13" t="inlineStr">
@@ -3889,7 +3889,7 @@
       <c r="H63" s="13" t="inlineStr"/>
       <c r="I63" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008122</t>
+          <t>voc4cat:0008122</t>
         </is>
       </c>
       <c r="J63" s="13" t="inlineStr">
@@ -3929,7 +3929,7 @@
       <c r="H64" s="13" t="inlineStr"/>
       <c r="I64" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008207</t>
+          <t>voc4cat:0008207</t>
         </is>
       </c>
       <c r="J64" s="13" t="inlineStr">
@@ -4005,7 +4005,7 @@
       <c r="H66" s="13" t="inlineStr"/>
       <c r="I66" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008206</t>
+          <t>voc4cat:0008206</t>
         </is>
       </c>
       <c r="J66" s="13" t="inlineStr">
@@ -4089,7 +4089,7 @@
       <c r="H68" s="13" t="inlineStr"/>
       <c r="I68" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008208</t>
+          <t>voc4cat:0008208</t>
         </is>
       </c>
       <c r="J68" s="13" t="inlineStr">
@@ -4162,7 +4162,7 @@
       <c r="H70" s="16" t="inlineStr"/>
       <c r="I70" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000055</t>
+          <t>voc4cat:0000055</t>
         </is>
       </c>
       <c r="J70" s="16" t="inlineStr">
@@ -4349,7 +4349,7 @@
       <c r="H75" s="13" t="inlineStr"/>
       <c r="I75" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000060</t>
+          <t>voc4cat:0000060</t>
         </is>
       </c>
       <c r="J75" s="13" t="inlineStr">
@@ -4425,7 +4425,7 @@
       <c r="H77" s="13" t="inlineStr"/>
       <c r="I77" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008123</t>
+          <t>voc4cat:0008123</t>
         </is>
       </c>
       <c r="J77" s="13" t="inlineStr">
@@ -4509,7 +4509,7 @@
       <c r="H79" s="16" t="inlineStr"/>
       <c r="I79" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000055</t>
+          <t>voc4cat:0000055</t>
         </is>
       </c>
       <c r="J79" s="16" t="inlineStr">
@@ -4550,7 +4550,7 @@
       <c r="H80" s="13" t="inlineStr"/>
       <c r="I80" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008116</t>
+          <t>voc4cat:0008116</t>
         </is>
       </c>
       <c r="J80" s="13" t="inlineStr">
@@ -4626,7 +4626,7 @@
       <c r="H82" s="13" t="inlineStr"/>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000056</t>
+          <t>voc4cat:0000056</t>
         </is>
       </c>
       <c r="J82" s="13" t="inlineStr">
@@ -4698,7 +4698,7 @@
       <c r="H84" s="16" t="inlineStr"/>
       <c r="I84" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007795</t>
+          <t>voc4cat:0007795</t>
         </is>
       </c>
       <c r="J84" s="16" t="inlineStr">
@@ -4779,7 +4779,7 @@
       <c r="H86" s="13" t="inlineStr"/>
       <c r="I86" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008203</t>
+          <t>voc4cat:0008203</t>
         </is>
       </c>
       <c r="J86" s="13" t="inlineStr">
@@ -4863,7 +4863,7 @@
       <c r="H88" s="13" t="inlineStr"/>
       <c r="I88" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008125</t>
+          <t>voc4cat:0008125</t>
         </is>
       </c>
       <c r="J88" s="13" t="inlineStr">
@@ -5087,7 +5087,7 @@
       <c r="H94" s="13" t="inlineStr"/>
       <c r="I94" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008126</t>
+          <t>voc4cat:0008126</t>
         </is>
       </c>
       <c r="J94" s="13" t="inlineStr">
@@ -5163,7 +5163,7 @@
       <c r="H96" s="13" t="inlineStr"/>
       <c r="I96" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008127</t>
+          <t>voc4cat:0008127</t>
         </is>
       </c>
       <c r="J96" s="13" t="inlineStr">
@@ -5243,7 +5243,7 @@
       <c r="H98" s="13" t="inlineStr"/>
       <c r="I98" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008128</t>
+          <t>voc4cat:0008128</t>
         </is>
       </c>
       <c r="J98" s="13" t="inlineStr">
@@ -5287,7 +5287,7 @@
       <c r="H99" s="13" t="inlineStr"/>
       <c r="I99" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008129</t>
+          <t>voc4cat:0008129</t>
         </is>
       </c>
       <c r="J99" s="13" t="inlineStr">
@@ -5331,7 +5331,7 @@
       <c r="H100" s="13" t="inlineStr"/>
       <c r="I100" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008130</t>
+          <t>voc4cat:0008130</t>
         </is>
       </c>
       <c r="J100" s="13" t="inlineStr">
@@ -5371,7 +5371,7 @@
       <c r="H101" s="13" t="inlineStr"/>
       <c r="I101" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008131</t>
+          <t>voc4cat:0008131</t>
         </is>
       </c>
       <c r="J101" s="13" t="inlineStr">
@@ -5447,7 +5447,7 @@
       <c r="H103" s="13" t="inlineStr"/>
       <c r="I103" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008204</t>
+          <t>voc4cat:0008204</t>
         </is>
       </c>
       <c r="J103" s="13" t="inlineStr">
@@ -5527,7 +5527,7 @@
       <c r="H105" s="13" t="inlineStr"/>
       <c r="I105" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008122</t>
+          <t>voc4cat:0008122</t>
         </is>
       </c>
       <c r="J105" s="13" t="inlineStr">
@@ -5567,7 +5567,7 @@
       <c r="H106" s="13" t="inlineStr"/>
       <c r="I106" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008207</t>
+          <t>voc4cat:0008207</t>
         </is>
       </c>
       <c r="J106" s="13" t="inlineStr">
@@ -5607,7 +5607,7 @@
       <c r="H107" s="13" t="inlineStr"/>
       <c r="I107" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008206</t>
+          <t>voc4cat:0008206</t>
         </is>
       </c>
       <c r="J107" s="13" t="inlineStr">
@@ -5655,7 +5655,7 @@
       <c r="H108" s="13" t="inlineStr"/>
       <c r="I108" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008208</t>
+          <t>voc4cat:0008208</t>
         </is>
       </c>
       <c r="J108" s="13" t="inlineStr">
@@ -5736,7 +5736,7 @@
       <c r="H110" s="13" t="inlineStr"/>
       <c r="I110" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000060</t>
+          <t>voc4cat:0000060</t>
         </is>
       </c>
       <c r="J110" s="13" t="inlineStr">
@@ -5776,7 +5776,7 @@
       <c r="H111" s="13" t="inlineStr"/>
       <c r="I111" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008123</t>
+          <t>voc4cat:0008123</t>
         </is>
       </c>
       <c r="J111" s="13" t="inlineStr">
@@ -5864,7 +5864,7 @@
       <c r="H113" s="13" t="inlineStr"/>
       <c r="I113" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008116</t>
+          <t>voc4cat:0008116</t>
         </is>
       </c>
       <c r="J113" s="13" t="inlineStr">
@@ -5904,7 +5904,7 @@
       <c r="H114" s="13" t="inlineStr"/>
       <c r="I114" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000056</t>
+          <t>voc4cat:0000056</t>
         </is>
       </c>
       <c r="J114" s="13" t="inlineStr">
@@ -6025,7 +6025,7 @@
       <c r="H117" s="13" t="inlineStr"/>
       <c r="I117" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008204</t>
+          <t>voc4cat:0008204</t>
         </is>
       </c>
       <c r="J117" s="13" t="inlineStr">
@@ -6189,7 +6189,7 @@
       <c r="H121" s="13" t="inlineStr"/>
       <c r="I121" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008122</t>
+          <t>voc4cat:0008122</t>
         </is>
       </c>
       <c r="J121" s="13" t="inlineStr">
@@ -6229,7 +6229,7 @@
       <c r="H122" s="13" t="inlineStr"/>
       <c r="I122" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008207</t>
+          <t>voc4cat:0008207</t>
         </is>
       </c>
       <c r="J122" s="13" t="inlineStr">
@@ -6269,7 +6269,7 @@
       <c r="H123" s="13" t="inlineStr"/>
       <c r="I123" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008206</t>
+          <t>voc4cat:0008206</t>
         </is>
       </c>
       <c r="J123" s="13" t="inlineStr">
@@ -6317,7 +6317,7 @@
       <c r="H124" s="13" t="inlineStr"/>
       <c r="I124" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008208</t>
+          <t>voc4cat:0008208</t>
         </is>
       </c>
       <c r="J124" s="13" t="inlineStr">
@@ -6446,7 +6446,7 @@
       <c r="H127" s="13" t="inlineStr"/>
       <c r="I127" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008113</t>
+          <t>voc4cat:0008113</t>
         </is>
       </c>
       <c r="J127" s="13" t="inlineStr">
@@ -6610,7 +6610,7 @@
       <c r="H131" s="13" t="inlineStr"/>
       <c r="I131" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000051</t>
+          <t>voc4cat:0000051</t>
         </is>
       </c>
       <c r="J131" s="13" t="inlineStr">
@@ -6694,7 +6694,7 @@
       <c r="H133" s="13" t="inlineStr"/>
       <c r="I133" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000050</t>
+          <t>voc4cat:0000050</t>
         </is>
       </c>
       <c r="J133" s="13" t="inlineStr">
@@ -6863,7 +6863,7 @@
       <c r="H137" s="13" t="inlineStr"/>
       <c r="I137" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J137" s="13" t="inlineStr">
@@ -7197,7 +7197,7 @@
       <c r="H145" s="13" t="inlineStr"/>
       <c r="I145" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000053</t>
+          <t>voc4cat:0000053</t>
         </is>
       </c>
       <c r="J145" s="13" t="inlineStr">
@@ -7309,7 +7309,7 @@
       <c r="H148" s="13" t="inlineStr"/>
       <c r="I148" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000051</t>
+          <t>voc4cat:0000051</t>
         </is>
       </c>
       <c r="J148" s="13" t="inlineStr">
@@ -7357,7 +7357,7 @@
       <c r="H149" s="13" t="inlineStr"/>
       <c r="I149" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000050</t>
+          <t>voc4cat:0000050</t>
         </is>
       </c>
       <c r="J149" s="13" t="inlineStr">
@@ -7453,7 +7453,7 @@
       <c r="H151" s="13" t="inlineStr"/>
       <c r="I151" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J151" s="13" t="inlineStr">
@@ -7830,7 +7830,7 @@
       <c r="H160" s="13" t="inlineStr"/>
       <c r="I160" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000051</t>
+          <t>voc4cat:0000051</t>
         </is>
       </c>
       <c r="J160" s="13" t="inlineStr">
@@ -7878,7 +7878,7 @@
       <c r="H161" s="13" t="inlineStr"/>
       <c r="I161" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000050</t>
+          <t>voc4cat:0000050</t>
         </is>
       </c>
       <c r="J161" s="13" t="inlineStr">
@@ -7974,7 +7974,7 @@
       <c r="H163" s="13" t="inlineStr"/>
       <c r="I163" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J163" s="13" t="inlineStr">
@@ -8056,7 +8056,7 @@
       <c r="H165" s="13" t="inlineStr"/>
       <c r="I165" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000024</t>
+          <t>voc4cat:0000024</t>
         </is>
       </c>
       <c r="J165" s="13" t="inlineStr">
@@ -8152,7 +8152,7 @@
       </c>
       <c r="I167" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000112</t>
+          <t>voc4cat:0000112</t>
         </is>
       </c>
       <c r="J167" s="13" t="inlineStr">
@@ -8192,7 +8192,7 @@
       <c r="H168" s="13" t="inlineStr"/>
       <c r="I168" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008123</t>
+          <t>voc4cat:0008123</t>
         </is>
       </c>
       <c r="J168" s="13" t="inlineStr">
@@ -8641,7 +8641,7 @@
       <c r="H179" s="13" t="inlineStr"/>
       <c r="I179" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008203</t>
+          <t>voc4cat:0008203</t>
         </is>
       </c>
       <c r="J179" s="13" t="inlineStr">
@@ -8689,7 +8689,7 @@
       <c r="H180" s="13" t="inlineStr"/>
       <c r="I180" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008125</t>
+          <t>voc4cat:0008125</t>
         </is>
       </c>
       <c r="J180" s="13" t="inlineStr">
@@ -8809,7 +8809,7 @@
       <c r="H183" s="13" t="inlineStr"/>
       <c r="I183" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008126</t>
+          <t>voc4cat:0008126</t>
         </is>
       </c>
       <c r="J183" s="13" t="inlineStr">
@@ -8849,7 +8849,7 @@
       <c r="H184" s="13" t="inlineStr"/>
       <c r="I184" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008127</t>
+          <t>voc4cat:0008127</t>
         </is>
       </c>
       <c r="J184" s="13" t="inlineStr">
@@ -8893,7 +8893,7 @@
       <c r="H185" s="13" t="inlineStr"/>
       <c r="I185" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008128</t>
+          <t>voc4cat:0008128</t>
         </is>
       </c>
       <c r="J185" s="13" t="inlineStr">
@@ -8937,7 +8937,7 @@
       <c r="H186" s="13" t="inlineStr"/>
       <c r="I186" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008129</t>
+          <t>voc4cat:0008129</t>
         </is>
       </c>
       <c r="J186" s="13" t="inlineStr">
@@ -8981,7 +8981,7 @@
       <c r="H187" s="13" t="inlineStr"/>
       <c r="I187" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008130</t>
+          <t>voc4cat:0008130</t>
         </is>
       </c>
       <c r="J187" s="13" t="inlineStr">
@@ -9021,7 +9021,7 @@
       <c r="H188" s="13" t="inlineStr"/>
       <c r="I188" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008131</t>
+          <t>voc4cat:0008131</t>
         </is>
       </c>
       <c r="J188" s="13" t="inlineStr">
@@ -9061,7 +9061,7 @@
       <c r="H189" s="13" t="inlineStr"/>
       <c r="I189" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008204</t>
+          <t>voc4cat:0008204</t>
         </is>
       </c>
       <c r="J189" s="13" t="inlineStr">
@@ -9105,7 +9105,7 @@
       <c r="H190" s="13" t="inlineStr"/>
       <c r="I190" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008122</t>
+          <t>voc4cat:0008122</t>
         </is>
       </c>
       <c r="J190" s="13" t="inlineStr">
@@ -9145,7 +9145,7 @@
       <c r="H191" s="13" t="inlineStr"/>
       <c r="I191" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008207</t>
+          <t>voc4cat:0008207</t>
         </is>
       </c>
       <c r="J191" s="13" t="inlineStr">
@@ -9185,7 +9185,7 @@
       <c r="H192" s="13" t="inlineStr"/>
       <c r="I192" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008206</t>
+          <t>voc4cat:0008206</t>
         </is>
       </c>
       <c r="J192" s="13" t="inlineStr">
@@ -9233,7 +9233,7 @@
       <c r="H193" s="13" t="inlineStr"/>
       <c r="I193" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008208</t>
+          <t>voc4cat:0008208</t>
         </is>
       </c>
       <c r="J193" s="13" t="inlineStr">
@@ -9314,7 +9314,7 @@
       <c r="H195" s="13" t="inlineStr"/>
       <c r="I195" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000060</t>
+          <t>voc4cat:0000060</t>
         </is>
       </c>
       <c r="J195" s="13" t="inlineStr">
@@ -9354,7 +9354,7 @@
       <c r="H196" s="13" t="inlineStr"/>
       <c r="I196" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008123</t>
+          <t>voc4cat:0008123</t>
         </is>
       </c>
       <c r="J196" s="13" t="inlineStr">
@@ -9442,7 +9442,7 @@
       <c r="H198" s="13" t="inlineStr"/>
       <c r="I198" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008116</t>
+          <t>voc4cat:0008116</t>
         </is>
       </c>
       <c r="J198" s="13" t="inlineStr">
@@ -9482,7 +9482,7 @@
       <c r="H199" s="13" t="inlineStr"/>
       <c r="I199" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000056</t>
+          <t>voc4cat:0000056</t>
         </is>
       </c>
       <c r="J199" s="13" t="inlineStr">
@@ -9695,7 +9695,7 @@
       <c r="H204" s="13" t="inlineStr"/>
       <c r="I204" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000051</t>
+          <t>voc4cat:0000051</t>
         </is>
       </c>
       <c r="J204" s="13" t="inlineStr">
@@ -9743,7 +9743,7 @@
       <c r="H205" s="13" t="inlineStr"/>
       <c r="I205" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000050</t>
+          <t>voc4cat:0000050</t>
         </is>
       </c>
       <c r="J205" s="13" t="inlineStr">
@@ -9839,7 +9839,7 @@
       <c r="H207" s="13" t="inlineStr"/>
       <c r="I207" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J207" s="13" t="inlineStr">
@@ -10088,7 +10088,7 @@
       <c r="H213" s="13" t="inlineStr"/>
       <c r="I213" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008122</t>
+          <t>voc4cat:0008122</t>
         </is>
       </c>
       <c r="J213" s="13" t="inlineStr">
@@ -10128,7 +10128,7 @@
       <c r="H214" s="13" t="inlineStr"/>
       <c r="I214" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008207</t>
+          <t>voc4cat:0008207</t>
         </is>
       </c>
       <c r="J214" s="13" t="inlineStr">
@@ -10168,7 +10168,7 @@
       <c r="H215" s="13" t="inlineStr"/>
       <c r="I215" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008206</t>
+          <t>voc4cat:0008206</t>
         </is>
       </c>
       <c r="J215" s="13" t="inlineStr">
@@ -10216,7 +10216,7 @@
       <c r="H216" s="13" t="inlineStr"/>
       <c r="I216" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008208</t>
+          <t>voc4cat:0008208</t>
         </is>
       </c>
       <c r="J216" s="13" t="inlineStr">
@@ -10297,7 +10297,7 @@
       <c r="H218" s="13" t="inlineStr"/>
       <c r="I218" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000060</t>
+          <t>voc4cat:0000060</t>
         </is>
       </c>
       <c r="J218" s="13" t="inlineStr">
@@ -10337,7 +10337,7 @@
       <c r="H219" s="13" t="inlineStr"/>
       <c r="I219" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008123</t>
+          <t>voc4cat:0008123</t>
         </is>
       </c>
       <c r="J219" s="13" t="inlineStr">
@@ -10425,7 +10425,7 @@
       <c r="H221" s="13" t="inlineStr"/>
       <c r="I221" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008116</t>
+          <t>voc4cat:0008116</t>
         </is>
       </c>
       <c r="J221" s="13" t="inlineStr">
@@ -10465,7 +10465,7 @@
       <c r="H222" s="13" t="inlineStr"/>
       <c r="I222" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000056</t>
+          <t>voc4cat:0000056</t>
         </is>
       </c>
       <c r="J222" s="13" t="inlineStr">
@@ -10501,7 +10501,7 @@
       <c r="H223" s="16" t="inlineStr"/>
       <c r="I223" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007031</t>
+          <t>voc4cat:0007031</t>
         </is>
       </c>
       <c r="J223" s="16" t="inlineStr">
@@ -11447,7 +11447,7 @@
       <c r="H245" s="13" t="inlineStr"/>
       <c r="I245" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000051</t>
+          <t>voc4cat:0000051</t>
         </is>
       </c>
       <c r="J245" s="13" t="inlineStr">
@@ -11495,7 +11495,7 @@
       <c r="H246" s="13" t="inlineStr"/>
       <c r="I246" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000050</t>
+          <t>voc4cat:0000050</t>
         </is>
       </c>
       <c r="J246" s="13" t="inlineStr">
@@ -11591,7 +11591,7 @@
       <c r="H248" s="13" t="inlineStr"/>
       <c r="I248" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J248" s="13" t="inlineStr">
@@ -11676,7 +11676,7 @@
       <c r="H250" s="13" t="inlineStr"/>
       <c r="I250" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000053</t>
+          <t>voc4cat:0000053</t>
         </is>
       </c>
       <c r="J250" s="13" t="inlineStr">
@@ -11756,7 +11756,7 @@
       <c r="H252" s="13" t="inlineStr"/>
       <c r="I252" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000051</t>
+          <t>voc4cat:0000051</t>
         </is>
       </c>
       <c r="J252" s="13" t="inlineStr">
@@ -11804,7 +11804,7 @@
       <c r="H253" s="13" t="inlineStr"/>
       <c r="I253" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000050</t>
+          <t>voc4cat:0000050</t>
         </is>
       </c>
       <c r="J253" s="13" t="inlineStr">
@@ -11900,7 +11900,7 @@
       <c r="H255" s="13" t="inlineStr"/>
       <c r="I255" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J255" s="13" t="inlineStr">
@@ -12217,7 +12217,7 @@
       <c r="H263" s="13" t="inlineStr"/>
       <c r="I263" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008127</t>
+          <t>voc4cat:0008127</t>
         </is>
       </c>
       <c r="J263" s="13" t="inlineStr">
@@ -12393,7 +12393,7 @@
       <c r="H267" s="13" t="inlineStr"/>
       <c r="I267" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008203</t>
+          <t>voc4cat:0008203</t>
         </is>
       </c>
       <c r="J267" s="13" t="inlineStr">
@@ -12525,7 +12525,7 @@
       <c r="H270" s="13" t="inlineStr"/>
       <c r="I270" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008123</t>
+          <t>voc4cat:0008123</t>
         </is>
       </c>
       <c r="J270" s="13" t="inlineStr">
@@ -12621,7 +12621,7 @@
       <c r="H272" s="13" t="inlineStr"/>
       <c r="I272" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J272" s="13" t="inlineStr">
@@ -12697,7 +12697,7 @@
       <c r="H274" s="13" t="inlineStr"/>
       <c r="I274" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008122</t>
+          <t>voc4cat:0008122</t>
         </is>
       </c>
       <c r="J274" s="13" t="inlineStr">
@@ -12737,7 +12737,7 @@
       <c r="H275" s="13" t="inlineStr"/>
       <c r="I275" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008207</t>
+          <t>voc4cat:0008207</t>
         </is>
       </c>
       <c r="J275" s="13" t="inlineStr">
@@ -12777,7 +12777,7 @@
       <c r="H276" s="13" t="inlineStr"/>
       <c r="I276" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008206</t>
+          <t>voc4cat:0008206</t>
         </is>
       </c>
       <c r="J276" s="13" t="inlineStr">
@@ -12825,7 +12825,7 @@
       <c r="H277" s="13" t="inlineStr"/>
       <c r="I277" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008208</t>
+          <t>voc4cat:0008208</t>
         </is>
       </c>
       <c r="J277" s="13" t="inlineStr">
@@ -12975,7 +12975,7 @@
       <c r="H281" s="13" t="inlineStr"/>
       <c r="I281" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000060</t>
+          <t>voc4cat:0000060</t>
         </is>
       </c>
       <c r="J281" s="13" t="inlineStr">
@@ -13015,7 +13015,7 @@
       <c r="H282" s="13" t="inlineStr"/>
       <c r="I282" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008123</t>
+          <t>voc4cat:0008123</t>
         </is>
       </c>
       <c r="J282" s="13" t="inlineStr">
@@ -13103,7 +13103,7 @@
       <c r="H284" s="13" t="inlineStr"/>
       <c r="I284" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008116</t>
+          <t>voc4cat:0008116</t>
         </is>
       </c>
       <c r="J284" s="13" t="inlineStr">
@@ -13143,7 +13143,7 @@
       <c r="H285" s="13" t="inlineStr"/>
       <c r="I285" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000056</t>
+          <t>voc4cat:0000056</t>
         </is>
       </c>
       <c r="J285" s="13" t="inlineStr">
@@ -13341,7 +13341,7 @@
       <c r="H4" s="13" t="inlineStr"/>
       <c r="I4" s="13" t="inlineStr">
         <is>
-          <t>AFP:0001159</t>
+          <t>allotrope.quality:0001159</t>
         </is>
       </c>
       <c r="J4" s="13" t="inlineStr">
@@ -13421,7 +13421,7 @@
       <c r="H6" s="16" t="inlineStr"/>
       <c r="I6" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000122</t>
+          <t>voc4cat:0000122</t>
         </is>
       </c>
       <c r="J6" s="16" t="inlineStr">
@@ -13462,7 +13462,7 @@
       <c r="H7" s="13" t="inlineStr"/>
       <c r="I7" s="13" t="inlineStr">
         <is>
-          <t>AFR:0000317</t>
+          <t>allotrope.result:0000317</t>
         </is>
       </c>
       <c r="J7" s="13" t="inlineStr">
@@ -13830,7 +13830,7 @@
       <c r="H17" s="13" t="inlineStr"/>
       <c r="I17" s="13" t="inlineStr">
         <is>
-          <t>AFR:0000950</t>
+          <t>allotrope.result:0000950</t>
         </is>
       </c>
       <c r="J17" s="13" t="inlineStr">
@@ -13914,7 +13914,7 @@
       <c r="H19" s="16" t="inlineStr"/>
       <c r="I19" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000108</t>
+          <t>voc4cat:0000108</t>
         </is>
       </c>
       <c r="J19" s="16" t="inlineStr">
@@ -13963,7 +13963,7 @@
       <c r="H20" s="13" t="inlineStr"/>
       <c r="I20" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J20" s="13" t="inlineStr">
@@ -14036,7 +14036,7 @@
       <c r="H22" s="16" t="inlineStr"/>
       <c r="I22" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000055</t>
+          <t>voc4cat:0000055</t>
         </is>
       </c>
       <c r="J22" s="16" t="inlineStr">
@@ -14625,7 +14625,7 @@
       <c r="H37" s="16" t="inlineStr"/>
       <c r="I37" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000286</t>
+          <t>voc4cat:0000286</t>
         </is>
       </c>
       <c r="J37" s="16" t="inlineStr">
@@ -14809,7 +14809,7 @@
       <c r="H41" s="13" t="inlineStr"/>
       <c r="I41" s="13" t="inlineStr">
         <is>
-          <t>AFR:0000950</t>
+          <t>allotrope.result:0000950</t>
         </is>
       </c>
       <c r="J41" s="13" t="inlineStr">
@@ -15013,7 +15013,7 @@
       <c r="H46" s="13" t="inlineStr"/>
       <c r="I46" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008123</t>
+          <t>voc4cat:0008123</t>
         </is>
       </c>
       <c r="J46" s="13" t="inlineStr">
@@ -15419,7 +15419,7 @@
       <c r="H56" s="13" t="inlineStr"/>
       <c r="I56" s="13" t="inlineStr">
         <is>
-          <t>AFR:0000950</t>
+          <t>allotrope.result:0000950</t>
         </is>
       </c>
       <c r="J56" s="13" t="inlineStr">
@@ -15719,7 +15719,7 @@
       <c r="H63" s="13" t="inlineStr"/>
       <c r="I63" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J63" s="13" t="inlineStr">
@@ -16414,7 +16414,7 @@
       <c r="H80" s="13" t="inlineStr"/>
       <c r="I80" s="13" t="inlineStr">
         <is>
-          <t>AFR:0000950</t>
+          <t>allotrope.result:0000950</t>
         </is>
       </c>
       <c r="J80" s="13" t="inlineStr">
@@ -16498,7 +16498,7 @@
       <c r="H82" s="13" t="inlineStr"/>
       <c r="I82" s="13" t="inlineStr">
         <is>
-          <t>AFP:0003721</t>
+          <t>allotrope.quality:0003721</t>
         </is>
       </c>
       <c r="J82" s="13" t="inlineStr">
@@ -16586,7 +16586,7 @@
       <c r="H84" s="13" t="inlineStr"/>
       <c r="I84" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J84" s="13" t="inlineStr">
@@ -17323,7 +17323,7 @@
       <c r="H103" s="13" t="inlineStr"/>
       <c r="I103" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J103" s="13" t="inlineStr">
@@ -17572,7 +17572,7 @@
       <c r="H109" s="13" t="inlineStr"/>
       <c r="I109" s="13" t="inlineStr">
         <is>
-          <t>AFR:0000950</t>
+          <t>allotrope.result:0000950</t>
         </is>
       </c>
       <c r="J109" s="13" t="inlineStr">
@@ -17808,7 +17808,7 @@
       <c r="H115" s="16" t="inlineStr"/>
       <c r="I115" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000069</t>
+          <t>voc4cat:0000069</t>
         </is>
       </c>
       <c r="J115" s="16" t="inlineStr">
@@ -17856,7 +17856,7 @@
       <c r="H116" s="13" t="inlineStr"/>
       <c r="I116" s="13" t="inlineStr">
         <is>
-          <t>AFR:0001594</t>
+          <t>allotrope.result:0001594</t>
         </is>
       </c>
       <c r="J116" s="13" t="inlineStr">
@@ -17940,7 +17940,7 @@
       <c r="H118" s="13" t="inlineStr"/>
       <c r="I118" s="13" t="inlineStr">
         <is>
-          <t>AFR:0001595</t>
+          <t>allotrope.result:0001595</t>
         </is>
       </c>
       <c r="J118" s="13" t="inlineStr">
@@ -18020,7 +18020,7 @@
       <c r="H120" s="13" t="inlineStr"/>
       <c r="I120" s="13" t="inlineStr">
         <is>
-          <t>AFR:0002226</t>
+          <t>allotrope.result:0002226</t>
         </is>
       </c>
       <c r="J120" s="13" t="inlineStr">
@@ -18184,7 +18184,7 @@
       <c r="H124" s="13" t="inlineStr"/>
       <c r="I124" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J124" s="13" t="inlineStr">
@@ -18336,7 +18336,7 @@
       <c r="H128" s="16" t="inlineStr"/>
       <c r="I128" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000073</t>
+          <t>voc4cat:0000073</t>
         </is>
       </c>
       <c r="J128" s="16" t="inlineStr">
@@ -18431,7 +18431,7 @@
       <c r="H130" s="13" t="inlineStr"/>
       <c r="I130" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007246</t>
+          <t>voc4cat:0007246</t>
         </is>
       </c>
       <c r="J130" s="13" t="inlineStr">
@@ -18731,7 +18731,7 @@
       <c r="H137" s="13" t="inlineStr"/>
       <c r="I137" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J137" s="13" t="inlineStr">
@@ -18799,7 +18799,7 @@
       <c r="H139" s="16" t="inlineStr"/>
       <c r="I139" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000078</t>
+          <t>voc4cat:0000078</t>
         </is>
       </c>
       <c r="J139" s="16" t="inlineStr">
@@ -19051,7 +19051,7 @@
       <c r="H145" s="13" t="inlineStr"/>
       <c r="I145" s="13" t="inlineStr">
         <is>
-          <t>AFR:0002226</t>
+          <t>allotrope.result:0002226</t>
         </is>
       </c>
       <c r="J145" s="13" t="inlineStr">
@@ -19087,7 +19087,7 @@
       <c r="H146" s="16" t="inlineStr"/>
       <c r="I146" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000075</t>
+          <t>voc4cat:0000075</t>
         </is>
       </c>
       <c r="J146" s="16" t="inlineStr">
@@ -19347,7 +19347,7 @@
       <c r="H152" s="13" t="inlineStr"/>
       <c r="I152" s="13" t="inlineStr">
         <is>
-          <t>AFR:0002226</t>
+          <t>allotrope.result:0002226</t>
         </is>
       </c>
       <c r="J152" s="13" t="inlineStr">
@@ -19479,7 +19479,7 @@
       <c r="H155" s="13" t="inlineStr"/>
       <c r="I155" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J155" s="13" t="inlineStr">
@@ -19913,7 +19913,7 @@
       <c r="H166" s="13" t="inlineStr"/>
       <c r="I166" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008116</t>
+          <t>voc4cat:0008116</t>
         </is>
       </c>
       <c r="J166" s="13" t="inlineStr">
@@ -20227,7 +20227,7 @@
       <c r="H174" s="13" t="inlineStr"/>
       <c r="I174" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008116</t>
+          <t>voc4cat:0008116</t>
         </is>
       </c>
       <c r="J174" s="13" t="inlineStr">
@@ -20468,7 +20468,7 @@
       <c r="H180" s="13" t="inlineStr"/>
       <c r="I180" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008116</t>
+          <t>voc4cat:0008116</t>
         </is>
       </c>
       <c r="J180" s="13" t="inlineStr">
@@ -20552,7 +20552,7 @@
       <c r="H182" s="16" t="inlineStr"/>
       <c r="I182" s="16" t="inlineStr">
         <is>
-          <t>ENM:0000064</t>
+          <t>enm:0000064</t>
         </is>
       </c>
       <c r="J182" s="16" t="inlineStr">
@@ -21440,7 +21440,7 @@
       <c r="H204" s="16" t="inlineStr"/>
       <c r="I204" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000079</t>
+          <t>voc4cat:0000079</t>
         </is>
       </c>
       <c r="J204" s="16" t="inlineStr">
@@ -21578,7 +21578,7 @@
       </c>
       <c r="I207" s="13" t="inlineStr">
         <is>
-          <t>AFQ:0000268</t>
+          <t>allotrope.quality:0000268</t>
         </is>
       </c>
       <c r="J207" s="13" t="inlineStr">
@@ -21626,7 +21626,7 @@
       <c r="H208" s="13" t="inlineStr"/>
       <c r="I208" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007246</t>
+          <t>voc4cat:0007246</t>
         </is>
       </c>
       <c r="J208" s="13" t="inlineStr">
@@ -21906,7 +21906,7 @@
       <c r="H215" s="13" t="inlineStr"/>
       <c r="I215" s="13" t="inlineStr">
         <is>
-          <t>AFR:0000950</t>
+          <t>allotrope.result:0000950</t>
         </is>
       </c>
       <c r="J215" s="13" t="inlineStr">
@@ -22026,7 +22026,7 @@
       <c r="H218" s="13" t="inlineStr"/>
       <c r="I218" s="13" t="inlineStr">
         <is>
-          <t>AFR:0002479</t>
+          <t>allotrope.result:0002479</t>
         </is>
       </c>
       <c r="J218" s="13" t="inlineStr">
@@ -22430,7 +22430,7 @@
       <c r="H228" s="13" t="inlineStr"/>
       <c r="I228" s="13" t="inlineStr">
         <is>
-          <t>AFR:0002479</t>
+          <t>allotrope.result:0002479</t>
         </is>
       </c>
       <c r="J228" s="13" t="inlineStr">
@@ -22646,7 +22646,7 @@
       </c>
       <c r="I233" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007213</t>
+          <t>voc4cat:0007213</t>
         </is>
       </c>
       <c r="J233" s="13" t="inlineStr">
@@ -22784,7 +22784,7 @@
       </c>
       <c r="I236" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007218</t>
+          <t>voc4cat:0007218</t>
         </is>
       </c>
       <c r="J236" s="13" t="inlineStr">
@@ -22824,7 +22824,7 @@
       <c r="H237" s="13" t="inlineStr"/>
       <c r="I237" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008123</t>
+          <t>voc4cat:0008123</t>
         </is>
       </c>
       <c r="J237" s="13" t="inlineStr">
@@ -22900,7 +22900,7 @@
       <c r="H239" s="13" t="inlineStr"/>
       <c r="I239" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007204</t>
+          <t>voc4cat:0007204</t>
         </is>
       </c>
       <c r="J239" s="13" t="inlineStr">
@@ -22944,7 +22944,7 @@
       <c r="H240" s="13" t="inlineStr"/>
       <c r="I240" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007202</t>
+          <t>voc4cat:0007202</t>
         </is>
       </c>
       <c r="J240" s="13" t="inlineStr">
@@ -22988,7 +22988,7 @@
       <c r="H241" s="13" t="inlineStr"/>
       <c r="I241" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007203</t>
+          <t>voc4cat:0007203</t>
         </is>
       </c>
       <c r="J241" s="13" t="inlineStr">
@@ -23164,7 +23164,7 @@
       <c r="H245" s="13" t="inlineStr"/>
       <c r="I245" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J245" s="13" t="inlineStr">
@@ -23332,7 +23332,7 @@
       </c>
       <c r="I249" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007239</t>
+          <t>voc4cat:0007239</t>
         </is>
       </c>
       <c r="J249" s="13" t="inlineStr">
@@ -23496,7 +23496,7 @@
       <c r="H253" s="13" t="inlineStr"/>
       <c r="I253" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007204</t>
+          <t>voc4cat:0007204</t>
         </is>
       </c>
       <c r="J253" s="13" t="inlineStr">
@@ -23540,7 +23540,7 @@
       <c r="H254" s="13" t="inlineStr"/>
       <c r="I254" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007202</t>
+          <t>voc4cat:0007202</t>
         </is>
       </c>
       <c r="J254" s="13" t="inlineStr">
@@ -23584,7 +23584,7 @@
       <c r="H255" s="13" t="inlineStr"/>
       <c r="I255" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007203</t>
+          <t>voc4cat:0007203</t>
         </is>
       </c>
       <c r="J255" s="13" t="inlineStr">
@@ -23724,7 +23724,7 @@
       <c r="H258" s="13" t="inlineStr"/>
       <c r="I258" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J258" s="13" t="inlineStr">
@@ -23848,7 +23848,7 @@
       <c r="H261" s="13" t="inlineStr"/>
       <c r="I261" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007246</t>
+          <t>voc4cat:0007246</t>
         </is>
       </c>
       <c r="J261" s="13" t="inlineStr">
@@ -23936,7 +23936,7 @@
       <c r="H263" s="13" t="inlineStr"/>
       <c r="I263" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000176</t>
+          <t>voc4cat:0000176</t>
         </is>
       </c>
       <c r="J263" s="13" t="inlineStr">
@@ -24636,7 +24636,7 @@
       <c r="H280" s="13" t="inlineStr"/>
       <c r="I280" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007246</t>
+          <t>voc4cat:0007246</t>
         </is>
       </c>
       <c r="J280" s="13" t="inlineStr">
@@ -25228,7 +25228,7 @@
       <c r="H294" s="13" t="inlineStr"/>
       <c r="I294" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008116</t>
+          <t>voc4cat:0008116</t>
         </is>
       </c>
       <c r="J294" s="13" t="inlineStr">
@@ -25616,7 +25616,7 @@
       <c r="H303" s="13" t="inlineStr"/>
       <c r="I303" s="13" t="inlineStr">
         <is>
-          <t>AFRL:0000011</t>
+          <t>allotrope.role:0000011</t>
         </is>
       </c>
       <c r="J303" s="13" t="inlineStr">
@@ -25933,7 +25933,7 @@
       <c r="H311" s="16" t="inlineStr"/>
       <c r="I311" s="16" t="inlineStr">
         <is>
-          <t>AFP:0000843</t>
+          <t>allotrope.quality:0000843</t>
         </is>
       </c>
       <c r="J311" s="16" t="inlineStr">
@@ -26141,7 +26141,7 @@
       <c r="H316" s="13" t="inlineStr"/>
       <c r="I316" s="13" t="inlineStr">
         <is>
-          <t>AFRL:0000011</t>
+          <t>allotrope.role:0000011</t>
         </is>
       </c>
       <c r="J316" s="13" t="inlineStr">
@@ -26597,7 +26597,7 @@
       <c r="H327" s="13" t="inlineStr"/>
       <c r="I327" s="13" t="inlineStr">
         <is>
-          <t>AFRL:0000011</t>
+          <t>allotrope.role:0000011</t>
         </is>
       </c>
       <c r="J327" s="13" t="inlineStr">
@@ -26999,7 +26999,7 @@
       <c r="H5" s="11" t="inlineStr"/>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007014</t>
+          <t>voc4cat:0007014</t>
         </is>
       </c>
       <c r="J5" s="11" t="inlineStr">
@@ -27017,10 +27017,10 @@
 CoreMeta4Cat#116 on whether this two-slot design (catalyst_type +
 catalyst_form) or PR #118's CatalystType class hierarchy should be
 the long-term mechanism -- kept as two enums here because the
-VOC4CAT terms show CatalystType conflates the regime axis
+voc4cat terms show CatalystType conflates the regime axis
 (Heterogeneous/Homogeneous/Bio/Electro/Photo) with the physical-form
 axis (ThinFilm/Bulk/Powdered/DepositedSample/Supported -- identical
-VOC4CAT ids to catalyst_form's permissible values), which are
+voc4cat ids to catalyst_form's permissible values), which are
 independent and often both apply to the same catalyst at once.</t>
         </is>
       </c>
@@ -27090,7 +27090,7 @@
       <c r="H7" s="11" t="inlineStr"/>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007009</t>
+          <t>voc4cat:0007009</t>
         </is>
       </c>
       <c r="J7" s="11" t="inlineStr">
@@ -27135,7 +27135,7 @@
       <c r="H8" s="13" t="inlineStr"/>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007032</t>
+          <t>voc4cat:0007032</t>
         </is>
       </c>
       <c r="J8" s="13" t="inlineStr">
@@ -27286,7 +27286,7 @@
       <c r="H12" s="13" t="inlineStr"/>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007809</t>
+          <t>voc4cat:0007809</t>
         </is>
       </c>
       <c r="J12" s="13" t="inlineStr">
@@ -27359,7 +27359,7 @@
       <c r="H14" s="16" t="inlineStr"/>
       <c r="I14" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000055</t>
+          <t>voc4cat:0000055</t>
         </is>
       </c>
       <c r="J14" s="16" t="inlineStr">
@@ -27404,7 +27404,7 @@
       <c r="H15" s="13" t="inlineStr"/>
       <c r="I15" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000118</t>
+          <t>voc4cat:0000118</t>
         </is>
       </c>
       <c r="J15" s="13" t="inlineStr">
@@ -31864,7 +31864,7 @@
       <c r="H128" s="16" t="inlineStr"/>
       <c r="I128" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007018</t>
+          <t>voc4cat:0007018</t>
         </is>
       </c>
       <c r="J128" s="16" t="inlineStr">
@@ -32189,7 +32189,7 @@
       <c r="H136" s="16" t="inlineStr"/>
       <c r="I136" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000193</t>
+          <t>voc4cat:0000193</t>
         </is>
       </c>
       <c r="J136" s="16" t="inlineStr">
@@ -32230,7 +32230,7 @@
       <c r="H137" s="11" t="inlineStr"/>
       <c r="I137" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007254</t>
+          <t>voc4cat:0007254</t>
         </is>
       </c>
       <c r="J137" s="11" t="inlineStr">
@@ -32272,7 +32272,7 @@
       <c r="H138" s="11" t="inlineStr"/>
       <c r="I138" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007255</t>
+          <t>voc4cat:0007255</t>
         </is>
       </c>
       <c r="J138" s="11" t="inlineStr">
@@ -32355,7 +32355,7 @@
       <c r="H140" s="13" t="inlineStr"/>
       <c r="I140" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007258</t>
+          <t>voc4cat:0007258</t>
         </is>
       </c>
       <c r="J140" s="13" t="inlineStr">
@@ -32432,7 +32432,7 @@
       <c r="H142" s="11" t="inlineStr"/>
       <c r="I142" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007259</t>
+          <t>voc4cat:0007259</t>
         </is>
       </c>
       <c r="J142" s="11" t="inlineStr">
@@ -32785,7 +32785,7 @@
       <c r="H151" s="16" t="inlineStr"/>
       <c r="I151" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007019</t>
+          <t>voc4cat:0007019</t>
         </is>
       </c>
       <c r="J151" s="16" t="inlineStr">
@@ -32826,7 +32826,7 @@
       <c r="H152" s="11" t="inlineStr"/>
       <c r="I152" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008114</t>
+          <t>voc4cat:0008114</t>
         </is>
       </c>
       <c r="J152" s="11" t="inlineStr">
@@ -32976,7 +32976,7 @@
       <c r="H156" s="11" t="inlineStr"/>
       <c r="I156" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000153</t>
+          <t>voc4cat:0000153</t>
         </is>
       </c>
       <c r="J156" s="11" t="inlineStr">
@@ -33125,7 +33125,7 @@
       <c r="H160" s="13" t="inlineStr"/>
       <c r="I160" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008115</t>
+          <t>voc4cat:0008115</t>
         </is>
       </c>
       <c r="J160" s="13" t="inlineStr">
@@ -33203,7 +33203,7 @@
       <c r="H162" s="13" t="inlineStr"/>
       <c r="I162" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008113</t>
+          <t>voc4cat:0008113</t>
         </is>
       </c>
       <c r="J162" s="13" t="inlineStr">
@@ -33523,7 +33523,7 @@
       <c r="H170" s="16" t="inlineStr"/>
       <c r="I170" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007102</t>
+          <t>voc4cat:0007102</t>
         </is>
       </c>
       <c r="J170" s="16" t="inlineStr">
@@ -33817,7 +33817,7 @@
       <c r="H178" s="11" t="inlineStr"/>
       <c r="I178" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008212</t>
+          <t>voc4cat:0008212</t>
         </is>
       </c>
       <c r="J178" s="11" t="inlineStr">
@@ -34248,7 +34248,7 @@
       <c r="H189" s="11" t="inlineStr"/>
       <c r="I189" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000156</t>
+          <t>voc4cat:0000156</t>
         </is>
       </c>
       <c r="J189" s="11" t="inlineStr">
@@ -34790,7 +34790,7 @@
       <c r="H203" s="11" t="inlineStr"/>
       <c r="I203" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008212</t>
+          <t>voc4cat:0008212</t>
         </is>
       </c>
       <c r="J203" s="11" t="inlineStr">
@@ -35327,7 +35327,7 @@
       <c r="H217" s="16" t="inlineStr"/>
       <c r="I217" s="16" t="inlineStr">
         <is>
-          <t>VOC4CAT:0000234</t>
+          <t>voc4cat:0000234</t>
         </is>
       </c>
       <c r="J217" s="16" t="inlineStr">
@@ -35839,7 +35839,7 @@
       <c r="H230" s="11" t="inlineStr"/>
       <c r="I230" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008212</t>
+          <t>voc4cat:0008212</t>
         </is>
       </c>
       <c r="J230" s="11" t="inlineStr">
@@ -35952,7 +35952,7 @@
       <c r="H233" s="11" t="inlineStr"/>
       <c r="I233" s="11" t="inlineStr">
         <is>
-          <t>VOC4CAT:0007021</t>
+          <t>voc4cat:0007021</t>
         </is>
       </c>
       <c r="J233" s="11" t="inlineStr">
@@ -36029,7 +36029,7 @@
       <c r="H235" s="13" t="inlineStr"/>
       <c r="I235" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008218</t>
+          <t>voc4cat:0008218</t>
         </is>
       </c>
       <c r="J235" s="13" t="inlineStr">
@@ -36070,7 +36070,7 @@
       <c r="H236" s="13" t="inlineStr"/>
       <c r="I236" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0008217</t>
+          <t>voc4cat:0008217</t>
         </is>
       </c>
       <c r="J236" s="13" t="inlineStr">
@@ -41764,7 +41764,7 @@
       <c r="H92" s="13" t="inlineStr"/>
       <c r="I92" s="13" t="inlineStr">
         <is>
-          <t>VOC4CAT:0005056</t>
+          <t>voc4cat:0005056</t>
         </is>
       </c>
       <c r="J92" s="13" t="inlineStr">

</xml_diff>